<commit_message>
13 evaluation tests for rotation
</commit_message>
<xml_diff>
--- a/Elements/extensions/textToScene/docs/textToScene_evaluation.xlsx
+++ b/Elements/extensions/textToScene/docs/textToScene_evaluation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yanni\Documents\GitHub\Elements\Elements\extensions\textToScene\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48182207-EBB7-465E-89A1-5342F5DF5D98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A1E2E66-F9B5-4F36-B01B-BA53E1D586E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Evaluation" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="241">
   <si>
     <t>#</t>
   </si>
@@ -573,13 +573,184 @@
   </si>
   <si>
     <t>In loaded scene with no recent changes fixxed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rotation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">rotate_object </t>
+  </si>
+  <si>
+    <t>cube_2</t>
+  </si>
+  <si>
+    <t>rotate the cube by 45 degrees</t>
+  </si>
+  <si>
+    <t>rotate the cube around the y axis</t>
+  </si>
+  <si>
+    <t>rotate the red cube around the y axis by 45 degrees</t>
+  </si>
+  <si>
+    <t>rotate the purple cube around the z axis by 30 degrees</t>
+  </si>
+  <si>
+    <t>turn the cube</t>
+  </si>
+  <si>
+    <t>spin the cube around y axis</t>
+  </si>
+  <si>
+    <t>rotate the cube by forty five degrees</t>
+  </si>
+  <si>
+    <t>rotate the sphere around y axis by 45 degrees</t>
+  </si>
+  <si>
+    <t>rotate</t>
+  </si>
+  <si>
+    <t>action_sequence + delete_object</t>
+  </si>
+  <si>
+    <t>rotate the cube</t>
+  </si>
+  <si>
+    <t>rotate the red cube</t>
+  </si>
+  <si>
+    <t>rotate the cube around q axis</t>
+  </si>
+  <si>
+    <t>selected cube rotates using the default rotation policy</t>
+  </si>
+  <si>
+    <t>selected red cube rotates using the default rotation policy</t>
+  </si>
+  <si>
+    <t>selected cube rotates by 45 degrees</t>
+  </si>
+  <si>
+    <t>selected cube rotates around the y axis</t>
+  </si>
+  <si>
+    <t>selected red cube rotates around the y axis by 45 degrees</t>
+  </si>
+  <si>
+    <t>selected purple cube rotates around the z axis by 30 degrees</t>
+  </si>
+  <si>
+    <t>command is normalized to rotate_object and the selected cube rotates</t>
+  </si>
+  <si>
+    <t>command is normalized to rotate_object and the selected cube rotates around the y axis</t>
+  </si>
+  <si>
+    <t>controlled validation failure for invalid rotation axis</t>
+  </si>
+  <si>
+    <t>command is normalized to a numeric angle or rejected cleanly if text angle parsing is unsupported</t>
+  </si>
+  <si>
+    <t>selected cube rotates by -45 degrees on the default or specified axis</t>
+  </si>
+  <si>
+    <t>selected sphere rotates around the y axis by 45 degrees</t>
+  </si>
+  <si>
+    <t>[controller] Parsed action: {'action': 'rotate_object', 'target': 'cube_1', 'axis': 'y', 'degrees': 45.0}</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> cube_1 -&gt; cube_1</t>
+  </si>
+  <si>
+    <t>Applied rotation: cube_1 axis=y degrees=45.0 rotation=[0.0, 45.0, 0.0]</t>
+  </si>
+  <si>
+    <t>{'action': 'rotate_object', 'target': 'red cube', 'axis': 'y', 'degrees': 45.0}</t>
+  </si>
+  <si>
+    <t>cube_2 axis=y degrees=45.0 rotation=[0.0, 45.0, 0.0]</t>
+  </si>
+  <si>
+    <t>rotate_object</t>
+  </si>
+  <si>
+    <t>{'action': 'rotate_object', 'target': 'cube_1', 'axis': 'y', 'degrees': 45.0}</t>
+  </si>
+  <si>
+    <t>Resolved target by id: cube_1 -&gt; cube_1</t>
+  </si>
+  <si>
+    <t>Applied rotation: cube_1 axis=y degrees=45.0 rotation=[0.0, 90.0, 0.0]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> by id: cube_1 -&gt; cube_1</t>
+  </si>
+  <si>
+    <t>Applied rotation: cube_1 axis=y degrees=45.0 rotation=[0.0, 135.0, 0.0]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> {'action': 'rotate_object', 'target': 'red cube', 'axis': 'y', 'degrees': 45.0}</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> by color+shape: red cube -&gt; cube_2</t>
+  </si>
+  <si>
+    <t>Applied rotation: cube_2 axis=y degrees=45.0 rotation=[0.0, 90.0, 0.0]</t>
+  </si>
+  <si>
+    <t>{'action': 'rotate_object', 'target': 'cube_1', 'axis': 'z', 'degrees': 30.0}</t>
+  </si>
+  <si>
+    <t>cube_1 -&gt; cube_1</t>
+  </si>
+  <si>
+    <t>Applied rotation: cube_1 axis=z degrees=30.0 rotation=[0.0, 135.0, 30.0]</t>
+  </si>
+  <si>
+    <t>Applied rotation: cube_1 axis=y degrees=45.0 rotation=[0.0, 225.0, 30.0]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Changed the axis to y instead of invalid axis  </t>
+  </si>
+  <si>
+    <t>Applied rotation: cube_1 axis=y degrees=45.0 rotation=[0.0, 315.0, 30.0]</t>
+  </si>
+  <si>
+    <t>{'action': 'rotate_object', 'target': 'sphere_1', 'axis': 'y', 'degrees': 45.0}</t>
+  </si>
+  <si>
+    <t>sphere_1 -&gt; sphere_1</t>
+  </si>
+  <si>
+    <t>sphere_1 axis=y degrees=45.0 rotation=[0.0, 45.0, 0.0]</t>
+  </si>
+  <si>
+    <t>any cube</t>
+  </si>
+  <si>
+    <t>rotate all objects -45 degrees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">all objects </t>
+  </si>
+  <si>
+    <t>Applying action_sequence step 1 of 3</t>
+  </si>
+  <si>
+    <t>action_sequence  + rotate_object</t>
+  </si>
+  <si>
+    <t>{'action': 'action_sequence', 'action_sequence': [{'action': 'rotate_object', 'target': 'cube_1', 'axis': 'y', 'degrees': -45.0}, {'action': 'rotate_object', 'target': 'cube_2', 'axis': 'y', 'degrees': -45.0}, {'action': 'rotate_object', 'target': 'sphere_1', 'axis': 'y', 'degrees': -45.0}]}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -649,8 +820,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="161"/>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -732,6 +911,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -860,7 +1051,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -886,28 +1077,15 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -917,27 +1095,15 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -956,9 +1122,6 @@
     <xf numFmtId="0" fontId="3" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -980,9 +1143,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -991,14 +1151,59 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1307,198 +1512,198 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K36"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K93"/>
+  <sheetFormatPr defaultRowHeight="45.6" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4" style="9" customWidth="1"/>
-    <col min="2" max="2" width="32" style="9" customWidth="1"/>
-    <col min="3" max="3" width="18" style="33" customWidth="1"/>
-    <col min="4" max="4" width="20" style="33" customWidth="1"/>
-    <col min="5" max="5" width="18" style="33" customWidth="1"/>
-    <col min="6" max="6" width="38" style="26" customWidth="1"/>
-    <col min="7" max="7" width="23.6640625" style="26" customWidth="1"/>
-    <col min="8" max="8" width="38" style="26" customWidth="1"/>
-    <col min="9" max="9" width="25.88671875" style="24" customWidth="1"/>
-    <col min="10" max="10" width="12" style="9" customWidth="1"/>
-    <col min="11" max="11" width="28" style="9" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="9"/>
+    <col min="1" max="1" width="4" style="43" customWidth="1"/>
+    <col min="2" max="2" width="32" style="31" customWidth="1"/>
+    <col min="3" max="3" width="18" style="43" customWidth="1"/>
+    <col min="4" max="4" width="20" style="43" customWidth="1"/>
+    <col min="5" max="5" width="18" style="43" customWidth="1"/>
+    <col min="6" max="6" width="38" style="42" customWidth="1"/>
+    <col min="7" max="7" width="23.6640625" style="43" customWidth="1"/>
+    <col min="8" max="8" width="38" style="31" customWidth="1"/>
+    <col min="9" max="9" width="25.88671875" style="31" customWidth="1"/>
+    <col min="10" max="10" width="12" style="52" customWidth="1"/>
+    <col min="11" max="11" width="28" style="43" customWidth="1"/>
+    <col min="12" max="16384" width="8.88671875" style="43"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="F1" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="18" t="s">
+      <c r="G1" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="H1" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="I1" s="18" t="s">
+      <c r="I1" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="J1" s="17" t="s">
+      <c r="J1" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="K1" s="17" t="s">
+      <c r="K1" s="12" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6">
         <v>1</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="37" t="s">
+      <c r="D2" s="27" t="s">
         <v>10</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="J2" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="K2" s="15"/>
-    </row>
-    <row r="3" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J2" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K2" s="6"/>
+    </row>
+    <row r="3" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="34" t="s">
+      <c r="C3" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="39" t="s">
+      <c r="D3" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="35" t="s">
+      <c r="E3" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="H3" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="I3" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="J3" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="K3" s="10"/>
-    </row>
-    <row r="4" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J3" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K3" s="8"/>
+    </row>
+    <row r="4" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6">
         <v>3</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="C4" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="40" t="s">
+      <c r="D4" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="36" t="s">
+      <c r="E4" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="37" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="H4" s="21" t="s">
+      <c r="H4" s="15" t="s">
         <v>93</v>
       </c>
       <c r="I4" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="J4" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="K4" s="15"/>
-    </row>
-    <row r="5" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J4" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K4" s="6"/>
+    </row>
+    <row r="5" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="8">
         <v>4</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="38" t="s">
+      <c r="D5" s="28" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="15" t="s">
+      <c r="G5" s="6" t="s">
         <v>74</v>
       </c>
       <c r="H5" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="I5" s="21" t="s">
+      <c r="I5" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="J5" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="K5" s="10"/>
-    </row>
-    <row r="6" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J5" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K5" s="8"/>
+    </row>
+    <row r="6" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6">
         <v>5</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="14" t="s">
         <v>9</v>
       </c>
       <c r="D6" s="6" t="s">
@@ -1507,64 +1712,64 @@
       <c r="E6" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="15" t="s">
+      <c r="G6" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="22" t="s">
+      <c r="H6" s="40" t="s">
         <v>91</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="J6" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="K6" s="15"/>
-    </row>
-    <row r="7" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J6" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K6" s="6"/>
+    </row>
+    <row r="7" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8">
         <v>6</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="23" t="s">
+      <c r="C7" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="10" t="s">
         <v>27</v>
       </c>
       <c r="E7" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="H7" s="24" t="s">
+      <c r="H7" s="31" t="s">
         <v>90</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="I7" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="J7" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="K7" s="10"/>
-    </row>
-    <row r="8" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J7" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K7" s="8"/>
+    </row>
+    <row r="8" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6">
         <v>7</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="C8" s="16" t="s">
         <v>26</v>
       </c>
       <c r="D8" s="6" t="s">
@@ -1573,27 +1778,27 @@
       <c r="E8" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="37" t="s">
         <v>32</v>
       </c>
-      <c r="G8" s="15" t="s">
+      <c r="G8" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="11" t="s">
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+      <c r="J8" s="46" t="s">
         <v>71</v>
       </c>
-      <c r="K8" s="15"/>
-    </row>
-    <row r="9" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="6">
+      <c r="K8" s="6"/>
+    </row>
+    <row r="9" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="8">
         <v>8</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="16" t="s">
         <v>26</v>
       </c>
       <c r="D9" s="8" t="s">
@@ -1602,10 +1807,10 @@
       <c r="E9" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="10" t="s">
         <v>101</v>
       </c>
       <c r="H9" s="7" t="s">
@@ -1614,19 +1819,19 @@
       <c r="I9" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="J9" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="K9" s="10"/>
-    </row>
-    <row r="10" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="8">
+      <c r="J9" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K9" s="8"/>
+    </row>
+    <row r="10" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="6">
         <v>9</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="17" t="s">
         <v>36</v>
       </c>
       <c r="D10" s="6" t="s">
@@ -1635,31 +1840,31 @@
       <c r="E10" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="G10" s="26" t="s">
+      <c r="G10" s="43" t="s">
         <v>37</v>
       </c>
-      <c r="H10" s="24" t="s">
+      <c r="H10" s="31" t="s">
         <v>88</v>
       </c>
-      <c r="I10" s="21" t="s">
+      <c r="I10" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="J10" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="K10" s="15"/>
-    </row>
-    <row r="11" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="6">
+      <c r="J10" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K10" s="6"/>
+    </row>
+    <row r="11" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="8">
         <v>10</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="17" t="s">
         <v>36</v>
       </c>
       <c r="D11" s="8" t="s">
@@ -1668,31 +1873,31 @@
       <c r="E11" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="G11" s="26" t="s">
+      <c r="G11" s="43" t="s">
         <v>37</v>
       </c>
-      <c r="H11" s="24" t="s">
+      <c r="H11" s="31" t="s">
         <v>95</v>
       </c>
       <c r="I11" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="J11" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="K11" s="10"/>
-    </row>
-    <row r="12" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="8">
+      <c r="J11" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K11" s="8"/>
+    </row>
+    <row r="12" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="6">
         <v>11</v>
       </c>
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="17" t="s">
         <v>36</v>
       </c>
       <c r="D12" s="6" t="s">
@@ -1701,31 +1906,31 @@
       <c r="E12" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="F12" s="37" t="s">
         <v>42</v>
       </c>
-      <c r="G12" s="26" t="s">
+      <c r="G12" s="43" t="s">
         <v>37</v>
       </c>
-      <c r="H12" s="15" t="s">
+      <c r="H12" s="11" t="s">
         <v>97</v>
       </c>
       <c r="I12" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="J12" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="K12" s="15"/>
-    </row>
-    <row r="13" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="6">
+      <c r="J12" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K12" s="6"/>
+    </row>
+    <row r="13" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="8">
         <v>12</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="27" t="s">
+      <c r="C13" s="18" t="s">
         <v>44</v>
       </c>
       <c r="D13" s="8" t="s">
@@ -1734,64 +1939,64 @@
       <c r="E13" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="G13" s="26" t="s">
+      <c r="G13" s="43" t="s">
         <v>45</v>
       </c>
-      <c r="H13" s="21" t="s">
+      <c r="H13" s="15" t="s">
         <v>100</v>
       </c>
       <c r="I13" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="J13" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="K13" s="10"/>
-    </row>
-    <row r="14" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="8">
+      <c r="J13" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K13" s="8"/>
+    </row>
+    <row r="14" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="6">
         <v>13</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="C14" s="27" t="s">
+      <c r="C14" s="18" t="s">
         <v>44</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="28" t="s">
+      <c r="E14" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="F14" s="21" t="s">
+      <c r="F14" s="39" t="s">
         <v>104</v>
       </c>
-      <c r="G14" s="26" t="s">
+      <c r="G14" s="43" t="s">
         <v>45</v>
       </c>
-      <c r="H14" s="15" t="s">
+      <c r="H14" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="I14" s="10" t="s">
+      <c r="I14" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="J14" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="K14" s="15"/>
-    </row>
-    <row r="15" spans="1:11" s="12" customFormat="1" ht="70.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="6">
+      <c r="J14" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K14" s="6"/>
+    </row>
+    <row r="15" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="8">
         <v>14</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="27" t="s">
+      <c r="C15" s="18" t="s">
         <v>44</v>
       </c>
       <c r="D15" s="8" t="s">
@@ -1800,31 +2005,31 @@
       <c r="E15" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="F15" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="G15" s="16" t="s">
-        <v>107</v>
-      </c>
-      <c r="H15" s="42" t="s">
+      <c r="G15" s="43" t="s">
+        <v>196</v>
+      </c>
+      <c r="H15" s="31" t="s">
         <v>108</v>
       </c>
       <c r="I15" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="J15" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="K15" s="10"/>
-    </row>
-    <row r="16" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J15" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K15" s="8"/>
+    </row>
+    <row r="16" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="6">
         <v>15</v>
       </c>
-      <c r="B16" s="15" t="s">
+      <c r="B16" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="C16" s="29" t="s">
+      <c r="C16" s="20" t="s">
         <v>52</v>
       </c>
       <c r="D16" s="6" t="s">
@@ -1833,31 +2038,31 @@
       <c r="E16" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="F16" s="15" t="s">
+      <c r="F16" s="37" t="s">
         <v>55</v>
       </c>
-      <c r="G16" s="15" t="s">
+      <c r="G16" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="H16" s="15" t="s">
+      <c r="H16" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="I16" s="21" t="s">
+      <c r="I16" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="J16" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="K16" s="15"/>
-    </row>
-    <row r="17" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J16" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K16" s="6"/>
+    </row>
+    <row r="17" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8">
         <v>16</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C17" s="29" t="s">
+      <c r="C17" s="20" t="s">
         <v>52</v>
       </c>
       <c r="D17" s="8" t="s">
@@ -1866,571 +2071,1205 @@
       <c r="E17" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="F17" s="10" t="s">
+      <c r="F17" s="38" t="s">
         <v>58</v>
       </c>
-      <c r="G17" s="15" t="s">
+      <c r="G17" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="H17" s="10" t="s">
+      <c r="H17" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="I17" s="10" t="s">
+      <c r="I17" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="J17" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="K17" s="10"/>
-    </row>
-    <row r="18" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J17" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K17" s="8"/>
+    </row>
+    <row r="18" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6">
         <v>17</v>
       </c>
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="C18" s="20" t="s">
         <v>52</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="E18" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="F18" s="15" t="s">
+      <c r="F18" s="37" t="s">
         <v>59</v>
       </c>
-      <c r="G18" s="15" t="s">
+      <c r="G18" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="H18" s="15" t="s">
+      <c r="H18" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="I18" s="10" t="s">
+      <c r="I18" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="J18" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="K18" s="21" t="s">
+      <c r="J18" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K18" s="19" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8">
         <v>18</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="C19" s="30" t="s">
+      <c r="C19" s="21" t="s">
         <v>61</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>62</v>
       </c>
       <c r="E19" s="8"/>
-      <c r="F19" s="10" t="s">
+      <c r="F19" s="38" t="s">
         <v>63</v>
       </c>
-      <c r="G19" s="10" t="s">
+      <c r="G19" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="H19" s="24" t="s">
+      <c r="H19" s="31" t="s">
         <v>121</v>
       </c>
-      <c r="I19" s="10"/>
-      <c r="J19" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="K19" s="10"/>
-    </row>
-    <row r="20" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I19" s="9"/>
+      <c r="J19" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K19" s="8"/>
+    </row>
+    <row r="20" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="6">
         <v>19</v>
       </c>
       <c r="B20" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="C20" s="30" t="s">
+      <c r="C20" s="21" t="s">
         <v>61</v>
       </c>
       <c r="D20" s="8" t="s">
         <v>62</v>
       </c>
       <c r="E20" s="8"/>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="38" t="s">
         <v>63</v>
       </c>
-      <c r="G20" s="10" t="s">
+      <c r="G20" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="H20" s="24" t="s">
+      <c r="H20" s="31" t="s">
         <v>123</v>
       </c>
-      <c r="I20" s="10"/>
-      <c r="J20" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="K20" s="10"/>
-    </row>
-    <row r="21" spans="1:11" ht="59.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I20" s="9"/>
+      <c r="J20" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K20" s="8"/>
+    </row>
+    <row r="21" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="8">
         <v>20</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="C21" s="31" t="s">
+      <c r="C21" s="22" t="s">
         <v>61</v>
       </c>
       <c r="D21" s="8" t="s">
         <v>127</v>
       </c>
       <c r="E21" s="8"/>
-      <c r="F21" s="10" t="s">
+      <c r="F21" s="38" t="s">
         <v>128</v>
       </c>
-      <c r="G21" s="10" t="s">
+      <c r="G21" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="H21" s="24" t="s">
+      <c r="H21" s="31" t="s">
         <v>129</v>
       </c>
-      <c r="I21" s="10"/>
-      <c r="J21" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="K21" s="10"/>
-    </row>
-    <row r="22" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I21" s="9"/>
+      <c r="J21" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K21" s="8"/>
+    </row>
+    <row r="22" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="6">
         <v>21</v>
       </c>
-      <c r="B22" s="15" t="s">
+      <c r="B22" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="C22" s="30" t="s">
+      <c r="C22" s="21" t="s">
         <v>61</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>48</v>
       </c>
       <c r="E22" s="6"/>
-      <c r="F22" s="15" t="s">
+      <c r="F22" s="37" t="s">
         <v>65</v>
       </c>
-      <c r="G22" s="21" t="s">
+      <c r="G22" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="H22" s="15" t="s">
+      <c r="H22" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="I22" s="15" t="s">
+      <c r="I22" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="J22" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="K22" s="15"/>
-    </row>
-    <row r="23" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="6">
+      <c r="J22" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K22" s="6"/>
+    </row>
+    <row r="23" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="8">
         <v>22</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C23" s="32" t="s">
+      <c r="C23" s="23" t="s">
         <v>66</v>
       </c>
       <c r="D23" s="8" t="s">
         <v>66</v>
       </c>
       <c r="E23" s="8"/>
-      <c r="F23" s="10" t="s">
+      <c r="F23" s="38" t="s">
         <v>132</v>
       </c>
-      <c r="G23" s="10" t="s">
+      <c r="G23" s="8" t="s">
         <v>131</v>
       </c>
       <c r="H23" s="7"/>
-      <c r="I23" s="10"/>
-      <c r="J23" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="K23" s="7" t="s">
+      <c r="I23" s="9"/>
+      <c r="J23" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K23" s="10" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="8">
+    <row r="24" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="6">
         <v>23</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C24" s="32" t="s">
+      <c r="C24" s="23" t="s">
         <v>66</v>
       </c>
       <c r="D24" s="8" t="s">
         <v>66</v>
       </c>
       <c r="E24" s="8"/>
-      <c r="F24" s="10" t="s">
+      <c r="F24" s="38" t="s">
         <v>67</v>
       </c>
-      <c r="G24" s="10" t="s">
+      <c r="G24" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="H24" s="10" t="s">
+      <c r="H24" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="I24" s="10" t="s">
+      <c r="I24" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="J24" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="K24" s="7" t="s">
+      <c r="J24" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K24" s="10" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="25" spans="1:11" s="16" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="15">
+    <row r="25" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="8">
         <v>24</v>
       </c>
       <c r="B25" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="C25" s="41" t="s">
+      <c r="C25" s="48" t="s">
         <v>137</v>
       </c>
       <c r="D25" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="E25" s="14" t="s">
+      <c r="E25" s="43" t="s">
         <v>138</v>
       </c>
-      <c r="F25" s="10" t="s">
+      <c r="F25" s="38" t="s">
         <v>139</v>
       </c>
-      <c r="G25" s="16" t="s">
+      <c r="G25" s="43" t="s">
         <v>166</v>
       </c>
-      <c r="H25" s="42" t="s">
+      <c r="H25" s="31" t="s">
         <v>75</v>
       </c>
-      <c r="I25" s="42"/>
-      <c r="J25" s="11" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" s="16" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="10">
+      <c r="J25" s="45" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="6">
         <v>25</v>
       </c>
       <c r="B26" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="C26" s="41" t="s">
+      <c r="C26" s="48" t="s">
         <v>141</v>
       </c>
       <c r="D26" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="E26" s="14" t="s">
+      <c r="E26" s="43" t="s">
         <v>138</v>
       </c>
-      <c r="F26" s="10" t="s">
+      <c r="F26" s="38" t="s">
         <v>143</v>
       </c>
-      <c r="G26" s="16" t="s">
+      <c r="G26" s="43" t="s">
         <v>150</v>
       </c>
-      <c r="H26" s="42" t="s">
+      <c r="H26" s="31" t="s">
         <v>167</v>
       </c>
-      <c r="I26" s="42"/>
-      <c r="J26" s="11" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" s="16" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="15">
+      <c r="J26" s="45" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="8">
         <v>26</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="C27" s="41" t="s">
+      <c r="C27" s="48" t="s">
         <v>141</v>
       </c>
       <c r="D27" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="E27" s="14" t="s">
+      <c r="E27" s="43" t="s">
         <v>138</v>
       </c>
-      <c r="F27" s="10" t="s">
+      <c r="F27" s="38" t="s">
         <v>144</v>
       </c>
-      <c r="G27" s="16" t="s">
+      <c r="G27" s="43" t="s">
         <v>150</v>
       </c>
-      <c r="H27" s="16" t="s">
+      <c r="H27" s="31" t="s">
         <v>168</v>
       </c>
-      <c r="I27" s="42" t="s">
+      <c r="I27" s="31" t="s">
         <v>169</v>
       </c>
-      <c r="J27" s="11" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" s="16" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="10">
+      <c r="J27" s="45" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="6">
         <v>27</v>
       </c>
-      <c r="B28" s="16" t="s">
+      <c r="B28" s="31" t="s">
         <v>145</v>
       </c>
-      <c r="C28" s="41" t="s">
+      <c r="C28" s="48" t="s">
         <v>141</v>
       </c>
       <c r="D28" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="E28" s="14" t="s">
+      <c r="E28" s="43" t="s">
         <v>138</v>
       </c>
-      <c r="F28" s="10" t="s">
+      <c r="F28" s="38" t="s">
         <v>146</v>
       </c>
-      <c r="G28" s="16" t="s">
+      <c r="G28" s="43" t="s">
         <v>150</v>
       </c>
-      <c r="H28" s="16" t="s">
+      <c r="H28" s="31" t="s">
         <v>171</v>
       </c>
-      <c r="I28" s="42"/>
-      <c r="J28" s="11" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" s="16" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="15">
+      <c r="J28" s="45" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="8">
         <v>28</v>
       </c>
-      <c r="B29" s="16" t="s">
+      <c r="B29" s="31" t="s">
         <v>173</v>
       </c>
-      <c r="C29" s="41" t="s">
+      <c r="C29" s="48" t="s">
         <v>141</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="E29" s="14" t="s">
+      <c r="E29" s="43" t="s">
         <v>138</v>
       </c>
-      <c r="F29" s="10" t="s">
+      <c r="F29" s="38" t="s">
         <v>155</v>
       </c>
-      <c r="G29" s="16" t="s">
+      <c r="G29" s="43" t="s">
         <v>150</v>
       </c>
-      <c r="H29" s="46" t="s">
+      <c r="H29" s="47" t="s">
         <v>172</v>
       </c>
-      <c r="I29" s="42"/>
-      <c r="J29" s="11" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" s="16" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="15">
+      <c r="J29" s="45" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="6">
         <v>29</v>
       </c>
       <c r="B30" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="C30" s="47" t="s">
+      <c r="C30" s="49" t="s">
         <v>148</v>
       </c>
       <c r="D30" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="E30" s="14" t="s">
+      <c r="E30" s="43" t="s">
         <v>152</v>
       </c>
-      <c r="F30" s="10" t="s">
+      <c r="F30" s="38" t="s">
         <v>153</v>
       </c>
-      <c r="G30" s="16" t="s">
+      <c r="G30" s="43" t="s">
         <v>174</v>
       </c>
-      <c r="H30" s="16" t="s">
+      <c r="H30" s="31" t="s">
         <v>175</v>
       </c>
-      <c r="I30" s="42"/>
-      <c r="J30" s="11" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" s="16" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="10">
+      <c r="J30" s="45" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="8">
         <v>30</v>
       </c>
       <c r="B31" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="C31" s="41" t="s">
+      <c r="C31" s="48" t="s">
         <v>141</v>
       </c>
-      <c r="D31" s="16" t="s">
+      <c r="D31" s="43" t="s">
         <v>176</v>
       </c>
-      <c r="E31" s="14" t="s">
+      <c r="E31" s="43" t="s">
         <v>151</v>
       </c>
-      <c r="F31" s="10" t="s">
+      <c r="F31" s="38" t="s">
         <v>154</v>
       </c>
-      <c r="G31" s="16" t="s">
+      <c r="G31" s="43" t="s">
         <v>176</v>
       </c>
-      <c r="I31" s="42"/>
-      <c r="J31" s="11" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" s="16" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="15">
+      <c r="J31" s="45" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="6">
         <v>31</v>
       </c>
       <c r="B32" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="C32" s="41" t="s">
+      <c r="C32" s="48" t="s">
         <v>141</v>
       </c>
-      <c r="D32" s="16" t="s">
+      <c r="D32" s="43" t="s">
         <v>176</v>
       </c>
-      <c r="E32" s="14" t="s">
+      <c r="E32" s="43" t="s">
         <v>151</v>
       </c>
-      <c r="F32" s="10" t="s">
+      <c r="F32" s="38" t="s">
         <v>157</v>
       </c>
-      <c r="G32" s="16" t="s">
+      <c r="G32" s="43" t="s">
         <v>176</v>
       </c>
-      <c r="I32" s="42"/>
-      <c r="J32" s="11" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" s="16" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="10">
+      <c r="J32" s="45" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="8">
         <v>32</v>
       </c>
       <c r="B33" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="C33" s="41" t="s">
+      <c r="C33" s="48" t="s">
         <v>141</v>
       </c>
-      <c r="D33" s="16" t="s">
+      <c r="D33" s="43" t="s">
         <v>142</v>
       </c>
-      <c r="E33" s="14" t="s">
+      <c r="E33" s="43" t="s">
         <v>151</v>
       </c>
-      <c r="F33" s="10" t="s">
+      <c r="F33" s="38" t="s">
         <v>159</v>
       </c>
-      <c r="G33" s="16" t="s">
+      <c r="G33" s="43" t="s">
         <v>142</v>
       </c>
-      <c r="H33" s="16" t="s">
+      <c r="H33" s="31" t="s">
         <v>177</v>
       </c>
-      <c r="I33" s="42"/>
-      <c r="J33" s="11" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" s="16" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="10">
+      <c r="J33" s="45" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="6">
         <v>33</v>
       </c>
       <c r="B34" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="C34" s="41" t="s">
+      <c r="C34" s="48" t="s">
         <v>141</v>
       </c>
       <c r="D34" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="E34" s="14" t="s">
+      <c r="E34" s="43" t="s">
         <v>162</v>
       </c>
-      <c r="F34" s="10" t="s">
+      <c r="F34" s="38" t="s">
         <v>161</v>
       </c>
-      <c r="G34" s="16" t="s">
+      <c r="G34" s="43" t="s">
         <v>142</v>
       </c>
-      <c r="H34" s="16" t="s">
+      <c r="H34" s="31" t="s">
         <v>178</v>
       </c>
-      <c r="I34" s="42"/>
-      <c r="J34" s="11" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" s="16" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="10">
+      <c r="J34" s="45" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="8">
         <v>34</v>
       </c>
       <c r="B35" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="C35" s="41" t="s">
+      <c r="C35" s="48" t="s">
         <v>141</v>
       </c>
       <c r="D35" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="E35" s="14" t="s">
+      <c r="E35" s="43" t="s">
         <v>151</v>
       </c>
-      <c r="F35" s="10" t="s">
+      <c r="F35" s="38" t="s">
         <v>165</v>
       </c>
-      <c r="G35" s="16" t="s">
+      <c r="G35" s="43" t="s">
         <v>107</v>
       </c>
-      <c r="H35" s="16" t="s">
+      <c r="H35" s="31" t="s">
         <v>179</v>
       </c>
-      <c r="I35" s="26" t="s">
+      <c r="I35" s="31" t="s">
         <v>180</v>
       </c>
-      <c r="J35" s="48" t="s">
+      <c r="J35" s="50" t="s">
         <v>181</v>
       </c>
-      <c r="K35" s="16" t="s">
+      <c r="K35" s="43" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B36"/>
+    <row r="36" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="6">
+        <v>35</v>
+      </c>
+      <c r="B36" s="35" t="s">
+        <v>197</v>
+      </c>
+      <c r="C36" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="D36" s="43" t="s">
+        <v>185</v>
+      </c>
+      <c r="E36" s="43" t="s">
+        <v>138</v>
+      </c>
+      <c r="F36" s="41" t="s">
+        <v>200</v>
+      </c>
+      <c r="G36" s="43" t="s">
+        <v>217</v>
+      </c>
+      <c r="H36" s="43" t="s">
+        <v>212</v>
+      </c>
+      <c r="I36" s="31" t="s">
+        <v>213</v>
+      </c>
+      <c r="J36" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K36" s="43" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="8">
+        <v>36</v>
+      </c>
+      <c r="B37" s="35" t="s">
+        <v>198</v>
+      </c>
+      <c r="C37" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="D37" s="43" t="s">
+        <v>185</v>
+      </c>
+      <c r="E37" s="43" t="s">
+        <v>186</v>
+      </c>
+      <c r="F37" s="41" t="s">
+        <v>201</v>
+      </c>
+      <c r="G37" s="43" t="s">
+        <v>217</v>
+      </c>
+      <c r="H37" s="31" t="s">
+        <v>215</v>
+      </c>
+      <c r="I37" s="31" t="s">
+        <v>94</v>
+      </c>
+      <c r="J37" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K37" s="43" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="6">
+        <v>37</v>
+      </c>
+      <c r="B38" s="35" t="s">
+        <v>187</v>
+      </c>
+      <c r="C38" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="D38" s="43" t="s">
+        <v>185</v>
+      </c>
+      <c r="E38" s="43" t="s">
+        <v>235</v>
+      </c>
+      <c r="F38" s="41" t="s">
+        <v>202</v>
+      </c>
+      <c r="G38" s="43" t="s">
+        <v>217</v>
+      </c>
+      <c r="H38" s="31" t="s">
+        <v>218</v>
+      </c>
+      <c r="I38" s="31" t="s">
+        <v>219</v>
+      </c>
+      <c r="J38" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K38" s="43" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="8">
+        <v>38</v>
+      </c>
+      <c r="B39" s="35" t="s">
+        <v>188</v>
+      </c>
+      <c r="C39" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="D39" s="43" t="s">
+        <v>185</v>
+      </c>
+      <c r="E39" s="43" t="s">
+        <v>235</v>
+      </c>
+      <c r="F39" s="41" t="s">
+        <v>203</v>
+      </c>
+      <c r="G39" s="43" t="s">
+        <v>217</v>
+      </c>
+      <c r="H39" s="31" t="s">
+        <v>218</v>
+      </c>
+      <c r="I39" s="31" t="s">
+        <v>221</v>
+      </c>
+      <c r="J39" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K39" s="43" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="6">
+        <v>39</v>
+      </c>
+      <c r="B40" s="35" t="s">
+        <v>189</v>
+      </c>
+      <c r="C40" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="D40" s="43" t="s">
+        <v>185</v>
+      </c>
+      <c r="E40" s="43" t="s">
+        <v>186</v>
+      </c>
+      <c r="F40" s="41" t="s">
+        <v>204</v>
+      </c>
+      <c r="G40" s="43" t="s">
+        <v>217</v>
+      </c>
+      <c r="H40" s="31" t="s">
+        <v>223</v>
+      </c>
+      <c r="I40" s="31" t="s">
+        <v>224</v>
+      </c>
+      <c r="J40" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K40" s="43" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="8">
+        <v>40</v>
+      </c>
+      <c r="B41" s="35" t="s">
+        <v>190</v>
+      </c>
+      <c r="C41" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="D41" s="43" t="s">
+        <v>185</v>
+      </c>
+      <c r="E41" s="43" t="s">
+        <v>138</v>
+      </c>
+      <c r="F41" s="41" t="s">
+        <v>205</v>
+      </c>
+      <c r="G41" s="43" t="s">
+        <v>217</v>
+      </c>
+      <c r="H41" s="31" t="s">
+        <v>226</v>
+      </c>
+      <c r="I41" s="31" t="s">
+        <v>227</v>
+      </c>
+      <c r="J41" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K41" s="43" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="6">
+        <v>41</v>
+      </c>
+      <c r="B42" s="35" t="s">
+        <v>191</v>
+      </c>
+      <c r="C42" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="D42" s="43" t="s">
+        <v>185</v>
+      </c>
+      <c r="E42" s="43" t="s">
+        <v>235</v>
+      </c>
+      <c r="F42" s="41" t="s">
+        <v>206</v>
+      </c>
+      <c r="G42" s="43" t="s">
+        <v>217</v>
+      </c>
+      <c r="H42" s="31" t="s">
+        <v>218</v>
+      </c>
+      <c r="I42" s="31" t="s">
+        <v>227</v>
+      </c>
+      <c r="J42" s="45" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="8">
+        <v>42</v>
+      </c>
+      <c r="B43" s="35" t="s">
+        <v>192</v>
+      </c>
+      <c r="C43" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="D43" s="43" t="s">
+        <v>185</v>
+      </c>
+      <c r="E43" s="43" t="s">
+        <v>235</v>
+      </c>
+      <c r="F43" s="41" t="s">
+        <v>207</v>
+      </c>
+      <c r="G43" s="43" t="s">
+        <v>217</v>
+      </c>
+      <c r="H43" s="31" t="s">
+        <v>218</v>
+      </c>
+      <c r="I43" s="31" t="s">
+        <v>227</v>
+      </c>
+      <c r="J43" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K43" s="43" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="6">
+        <v>43</v>
+      </c>
+      <c r="B44" s="35" t="s">
+        <v>199</v>
+      </c>
+      <c r="C44" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="D44" s="43" t="s">
+        <v>185</v>
+      </c>
+      <c r="E44" s="43" t="s">
+        <v>235</v>
+      </c>
+      <c r="F44" s="41" t="s">
+        <v>208</v>
+      </c>
+      <c r="G44" s="43" t="s">
+        <v>217</v>
+      </c>
+      <c r="H44" s="31" t="s">
+        <v>218</v>
+      </c>
+      <c r="I44" s="31" t="s">
+        <v>227</v>
+      </c>
+      <c r="J44" s="50" t="s">
+        <v>181</v>
+      </c>
+      <c r="K44" s="43" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="8">
+        <v>44</v>
+      </c>
+      <c r="B45" s="35" t="s">
+        <v>193</v>
+      </c>
+      <c r="C45" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="D45" s="43" t="s">
+        <v>185</v>
+      </c>
+      <c r="E45" s="43" t="s">
+        <v>235</v>
+      </c>
+      <c r="F45" s="41" t="s">
+        <v>209</v>
+      </c>
+      <c r="G45" s="43" t="s">
+        <v>217</v>
+      </c>
+      <c r="H45" s="31" t="s">
+        <v>218</v>
+      </c>
+      <c r="I45" s="31" t="s">
+        <v>227</v>
+      </c>
+      <c r="J45" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K45" s="43" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="129" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="6">
+        <v>45</v>
+      </c>
+      <c r="B46" s="35" t="s">
+        <v>236</v>
+      </c>
+      <c r="C46" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="D46" s="43" t="s">
+        <v>185</v>
+      </c>
+      <c r="E46" s="43" t="s">
+        <v>237</v>
+      </c>
+      <c r="F46" s="41" t="s">
+        <v>210</v>
+      </c>
+      <c r="G46" s="43" t="s">
+        <v>239</v>
+      </c>
+      <c r="H46" s="31" t="s">
+        <v>240</v>
+      </c>
+      <c r="I46" s="31" t="s">
+        <v>238</v>
+      </c>
+      <c r="J46" s="45" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="8">
+        <v>46</v>
+      </c>
+      <c r="B47" s="35" t="s">
+        <v>194</v>
+      </c>
+      <c r="C47" s="51" t="s">
+        <v>184</v>
+      </c>
+      <c r="D47" s="43" t="s">
+        <v>185</v>
+      </c>
+      <c r="E47" s="43" t="s">
+        <v>162</v>
+      </c>
+      <c r="F47" s="41" t="s">
+        <v>211</v>
+      </c>
+      <c r="G47" s="43" t="s">
+        <v>217</v>
+      </c>
+      <c r="H47" s="31" t="s">
+        <v>232</v>
+      </c>
+      <c r="I47" s="31" t="s">
+        <v>233</v>
+      </c>
+      <c r="J47" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="K47" s="43" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="6">
+        <v>47</v>
+      </c>
+      <c r="J48" s="45"/>
+    </row>
+    <row r="49" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="8">
+        <v>48</v>
+      </c>
+      <c r="J49" s="45"/>
+    </row>
+    <row r="50" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="6">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="8">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="6">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="8">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="6">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="8">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="6">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="8">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="6">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="8">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="6">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="8">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="6">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="8">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="6">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="8">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="6">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="8">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="6">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="8">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="6">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="8">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="6">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="8">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="6">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="8">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="6">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="8">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="6">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="8">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="6">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="8">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="6">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="8">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="6">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="8">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="6">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="8">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="6">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="8">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="6">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="8">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="6">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="8">
+        <v>92</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="10" type="noConversion"/>
@@ -2440,7 +3279,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2448,12 +3287,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="2" spans="1:5" ht="7.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -2487,7 +3326,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="3">
-        <f t="shared" ref="E4:E12" si="0">IF(B4=0,"",C4/B4)</f>
+        <f t="shared" ref="E4:E13" si="0">IF(B4=0,"",C4/B4)</f>
         <v>1</v>
       </c>
     </row>
@@ -2601,12 +3440,12 @@
         <v>0</v>
       </c>
       <c r="E10" s="3">
-        <f t="shared" si="0"/>
+        <f>IF(B10=0,"",C10/B10)</f>
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="43" t="s">
+      <c r="A11" s="32" t="s">
         <v>137</v>
       </c>
       <c r="B11" s="2">
@@ -2619,27 +3458,47 @@
         <v>1</v>
       </c>
       <c r="E11" s="3">
+        <f>IF(B11=0,"",C11/B11)</f>
+        <v>0.90909090909090906</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="32" t="s">
+        <v>195</v>
+      </c>
+      <c r="B12" s="2">
+        <v>12</v>
+      </c>
+      <c r="C12" s="2">
+        <v>11</v>
+      </c>
+      <c r="D12" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+      <c r="E12" s="3">
+        <f>IF(B12=0,"",C12/B12)</f>
+        <v>0.91666666666666663</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B12" s="4">
-        <f>SUM(B4:B11)</f>
-        <v>34</v>
-      </c>
-      <c r="C12" s="4">
-        <f>SUM(C4:C11)</f>
-        <v>32</v>
-      </c>
-      <c r="D12" s="4">
-        <v>2</v>
-      </c>
-      <c r="E12" s="5">
+      <c r="B13" s="4">
+        <f>SUM(B4:B12)</f>
+        <v>46</v>
+      </c>
+      <c r="C13" s="4">
+        <f>SUM(C4:C12)</f>
+        <v>43</v>
+      </c>
+      <c r="D13" s="4">
+        <f>SUM(D4:D12)</f>
+        <v>3</v>
+      </c>
+      <c r="E13" s="5">
         <f t="shared" si="0"/>
-        <v>0.94117647058823528</v>
+        <v>0.93478260869565222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>